<commit_message>
feat(loop): AnyLogic integer-field rounding + landbridge→ViaRott mapping fix; operator console .xlsx upload + fixed all20 scope
- manual_worklist.py: 27 Integer-typed factors rounded; 8 percentage factors
  keep decimals (spec.md §7 item 20). NA/A_{Im,Ex}_LB now map to Vol*ViaRott
  fields, NO_ANYLOGIC_EQUIVALENT 7→3 (item 23).
- operator_api.ingest_round: accepts base64 file bytes + filename, magic-number
  sniffs .xlsx/.xls, write_bytes under real extension (item 21).
- operator console: KPI scope fixed to all20; file picker accepts .csv/.xlsx.
- rounds: round_20260906_090349 ingested (+10, browser-automation route,
  4 KPIs only) → 179 rows; round_20260906_103618 exported/pending; two pending
  rounds' worklists regenerated with corrected rounding + headers.
- spec.md §7 items 20-23. 172 tests pass.
</commit_message>
<xml_diff>
--- a/experimenting_ml/docs/anylogic/AnyLogic_Manual_Worklist_DEMO.xlsx
+++ b/experimenting_ml/docs/anylogic/AnyLogic_Manual_Worklist_DEMO.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="run_2026_09_01_001" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="run_2026_09_01_002" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_2026_09_01_001" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_2026_09_01_002" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,49 +475,49 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - NA_Im_LB</t>
+          <t xml:space="preserve">  - A_Ex_LB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - NA_Ex_LB</t>
+          <t xml:space="preserve">  - A_Im_LB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A_Im_LB</t>
+          <t xml:space="preserve">  - NA_Ex_LB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A_Ex_LB</t>
+          <t xml:space="preserve">  - NA_Im_LB</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Pct_NA_OB_Green</t>
+          <t xml:space="preserve">  - Pct_A_OB_Red</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Pct_NA_OB_Red</t>
+          <t xml:space="preserve">  - Pct_NA_OB_Green</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Pct_A_OB_Red</t>
+          <t xml:space="preserve">  - Pct_NA_OB_Red</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79.3</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>135.85</v>
+        <v>136</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>79.95</v>
+        <v>80</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.24</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.12</v>
+        <v>2</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38.61</v>
+        <v>39</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>17.55</v>
+        <v>18</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>112.24</v>
+        <v>112</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>70486.92999999996</v>
+        <v>70487</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1893818.61</v>
+        <v>1893819</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>119461.93</v>
+        <v>119462</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>127676.22</v>
+        <v>127676</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
@@ -1242,7 +1242,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2535484.5</v>
+        <v>2535484</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>301281.22</v>
+        <v>301281</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>211583.9999999999</v>
+        <v>211584</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4832049.6</v>
+        <v>4832050</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>469583.9999999999</v>
+        <v>469584</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>265267.2</v>
+        <v>265267</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5507308.8</v>
+        <v>5507309</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>488267.2</v>
+        <v>488267</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>82.96000000000001</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>142.12</v>
+        <v>142</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
@@ -2763,7 +2763,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>83.64</v>
+        <v>84</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -2778,7 +2778,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -2808,7 +2808,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -2868,7 +2868,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>39.6</v>
+        <v>40</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -3168,7 +3168,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>56.4</v>
+        <v>56</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>56.4</v>
+        <v>56</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>56.4</v>
+        <v>56</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
@@ -3213,7 +3213,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>56.4</v>
+        <v>56</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -3228,7 +3228,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>56.4</v>
+        <v>56</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -3243,7 +3243,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>56.4</v>
+        <v>56</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>53.25</v>
+        <v>53</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>86.61999999999999</v>
+        <v>87</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>20731.45000000002</v>
+        <v>20731</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2612163.6</v>
+        <v>2612164</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
@@ -3318,7 +3318,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>69706.45000000001</v>
+        <v>69706</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>127676.22</v>
+        <v>127676</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>301281.22</v>
+        <v>301281</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
@@ -3378,7 +3378,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>222163.2</v>
+        <v>222163</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>480163.2</v>
+        <v>480163</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>180863.9999999999</v>
+        <v>180864</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>403863.9999999999</v>
+        <v>403864</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>

</xml_diff>